<commit_message>
Add Page: Project Request
</commit_message>
<xml_diff>
--- a/public/files/template-import-leads.xlsx
+++ b/public/files/template-import-leads.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alsaskar Mirando\Documents\PT Saskardigital Solusi Indonesia\Projek\saskardigital\frontend\public\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alsaskar Mirando\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{43DB4955-0350-4E9F-9B2A-7DDFDAAD6DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C4C259-0A7A-4013-AFEA-507F8C79FD5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="21270" yWindow="780" windowWidth="21600" windowHeight="11385" xr2:uid="{B2EE394A-CC8E-4891-8EA0-DE060CD5C853}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Nama Lengkap</t>
   </si>
@@ -55,6 +55,21 @@
   </si>
   <si>
     <t>irsyadassegaf@gmail.com</t>
+  </si>
+  <si>
+    <t>testing notes</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>facebook ads</t>
+  </si>
+  <si>
+    <t>organic</t>
+  </si>
+  <si>
+    <t>referall</t>
   </si>
 </sst>
 </file>
@@ -440,17 +455,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E3CDA8F-59A2-462C-B84F-F7C97939C65D}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
     <col min="2" max="2" width="36.140625" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" customWidth="1"/>
-    <col min="4" max="4" width="27.140625" customWidth="1"/>
-    <col min="5" max="5" width="9.28515625" customWidth="1"/>
+    <col min="3" max="4" width="22.140625" customWidth="1"/>
+    <col min="5" max="5" width="27.140625" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -461,10 +476,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -474,9 +492,12 @@
       <c r="C2" s="2">
         <v>89694824154</v>
       </c>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -486,9 +507,12 @@
       <c r="C3" s="2">
         <v>89338438383</v>
       </c>
-      <c r="D3" s="2"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -498,103 +522,124 @@
       <c r="C4" s="2">
         <v>89483839294</v>
       </c>
-      <c r="D4" s="2"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" s="2"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E8" s="2"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E11" s="2"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E12" s="2"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E14" s="2"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E18" s="2"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Add Status Leads: Contacted & Import Leads Sosial Media
</commit_message>
<xml_diff>
--- a/public/files/template-import-leads.xlsx
+++ b/public/files/template-import-leads.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alsaskar Mirando\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alsaskar Mirando\Documents\PT Saskardigital Solusi Indonesia\Projek\saskardigital\frontend\public\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C4C259-0A7A-4013-AFEA-507F8C79FD5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2CC55BA-C844-4383-B92F-69DF388B46D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21270" yWindow="780" windowWidth="21600" windowHeight="11385" xr2:uid="{B2EE394A-CC8E-4891-8EA0-DE060CD5C853}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{B2EE394A-CC8E-4891-8EA0-DE060CD5C853}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Nama Lengkap</t>
   </si>
@@ -42,34 +42,46 @@
     <t>Alsaskar Mirando</t>
   </si>
   <si>
-    <t>alsaskarmirando@gmail.com</t>
-  </si>
-  <si>
     <t>Bintang Algaza</t>
   </si>
   <si>
-    <t>bintangalgaza@gmail.com</t>
-  </si>
-  <si>
     <t>Irsyad Assegaf</t>
   </si>
   <si>
-    <t>irsyadassegaf@gmail.com</t>
-  </si>
-  <si>
     <t>testing notes</t>
   </si>
   <si>
     <t>Source</t>
   </si>
   <si>
-    <t>facebook ads</t>
-  </si>
-  <si>
-    <t>organic</t>
-  </si>
-  <si>
-    <t>referall</t>
+    <t>Google Maps</t>
+  </si>
+  <si>
+    <t>Organic</t>
+  </si>
+  <si>
+    <t>Google Ads</t>
+  </si>
+  <si>
+    <t>Sosial Media</t>
+  </si>
+  <si>
+    <t>IG: @alsaskar</t>
+  </si>
+  <si>
+    <t>IG: @bintang</t>
+  </si>
+  <si>
+    <t>IG: @irsyad</t>
+  </si>
+  <si>
+    <t>irsyadassegaf-edit@gmail.com</t>
+  </si>
+  <si>
+    <t>bintangalgaza-edit@gmail.com</t>
+  </si>
+  <si>
+    <t>alsaskarmirando-edit@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -455,17 +467,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E3CDA8F-59A2-462C-B84F-F7C97939C65D}">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
     <col min="2" max="2" width="36.140625" customWidth="1"/>
-    <col min="3" max="4" width="22.140625" customWidth="1"/>
-    <col min="5" max="5" width="27.140625" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" customWidth="1"/>
+    <col min="3" max="5" width="22.140625" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" customWidth="1"/>
+    <col min="7" max="7" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -476,170 +488,198 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C2" s="2">
         <v>89694824154</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C3" s="2">
         <v>89338438383</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C4" s="2">
         <v>89483839294</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12" s="2"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14" s="2"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15" s="2"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17" s="2"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" s="2"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" s="2"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>